<commit_message>
Temporal final df of sobol samples-  so far 3330 samples
</commit_message>
<xml_diff>
--- a/data/raw/sobol_sensitivity_analysis_lhs_500.xlsx
+++ b/data/raw/sobol_sensitivity_analysis_lhs_500.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\kju10\Documents\LMU-STATISTICS &amp; DATA SCIENCE MASTER\WS2425\Consulting\project\Sensitivity-Analysis-and-Surrogate-Modeling-of-PEM-Fuel-Cells\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EBCE864-F37E-4964-B73A-A37336C7F9FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC90A865-8087-402C-817C-05003D4E4490}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -216,7 +216,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -262,6 +262,24 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -457,7 +475,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -518,6 +536,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3208,127 +3235,127 @@
         <v>45</v>
       </c>
       <c r="B15" s="1">
-        <f>SUM(B2:B14)</f>
+        <f t="shared" ref="B15:AF15" si="0">SUM(B2:B14)</f>
         <v>3.4411867871715898</v>
       </c>
       <c r="C15" s="1">
-        <f>SUM(C2:C14)</f>
+        <f t="shared" si="0"/>
         <v>3.9696331410487145</v>
       </c>
       <c r="D15" s="1">
-        <f>SUM(D2:D14)</f>
+        <f t="shared" si="0"/>
         <v>4.0472648938866573</v>
       </c>
       <c r="E15" s="1">
-        <f>SUM(E2:E14)</f>
+        <f t="shared" si="0"/>
         <v>4.0131345004848287</v>
       </c>
       <c r="F15" s="1">
-        <f>SUM(F2:F14)</f>
+        <f t="shared" si="0"/>
         <v>3.9345906767954713</v>
       </c>
       <c r="G15" s="1">
-        <f>SUM(G2:G14)</f>
+        <f t="shared" si="0"/>
         <v>3.8427151722682127</v>
       </c>
       <c r="H15" s="1">
-        <f>SUM(H2:H14)</f>
+        <f t="shared" si="0"/>
         <v>3.7235030008513794</v>
       </c>
       <c r="I15" s="1">
-        <f>SUM(I2:I14)</f>
+        <f t="shared" si="0"/>
         <v>3.5913064519361004</v>
       </c>
       <c r="J15" s="1">
-        <f>SUM(J2:J14)</f>
+        <f t="shared" si="0"/>
         <v>3.4714332900401308</v>
       </c>
       <c r="K15" s="1">
-        <f>SUM(K2:K14)</f>
+        <f t="shared" si="0"/>
         <v>3.3585608932991451</v>
       </c>
       <c r="L15" s="1">
-        <f>SUM(L2:L14)</f>
+        <f t="shared" si="0"/>
         <v>3.2586298146534989</v>
       </c>
       <c r="M15" s="1">
-        <f>SUM(M2:M14)</f>
+        <f t="shared" si="0"/>
         <v>3.1617962464575542</v>
       </c>
       <c r="N15" s="1">
-        <f>SUM(N2:N14)</f>
+        <f t="shared" si="0"/>
         <v>3.0969455693430281</v>
       </c>
       <c r="O15" s="1">
-        <f>SUM(O2:O14)</f>
+        <f t="shared" si="0"/>
         <v>3.0263022806998476</v>
       </c>
       <c r="P15" s="1">
-        <f>SUM(P2:P14)</f>
+        <f t="shared" si="0"/>
         <v>2.9353473069429437</v>
       </c>
       <c r="Q15" s="1">
-        <f>SUM(Q2:Q14)</f>
+        <f t="shared" si="0"/>
         <v>2.8576286538656825</v>
       </c>
       <c r="R15" s="1">
-        <f>SUM(R2:R14)</f>
+        <f t="shared" si="0"/>
         <v>2.8030980562257981</v>
       </c>
       <c r="S15" s="1">
-        <f>SUM(S2:S14)</f>
+        <f t="shared" si="0"/>
         <v>2.8318150984283572</v>
       </c>
       <c r="T15" s="1">
-        <f>SUM(T2:T14)</f>
+        <f t="shared" si="0"/>
         <v>2.7716811822097727</v>
       </c>
       <c r="U15" s="1">
-        <f>SUM(U2:U14)</f>
+        <f t="shared" si="0"/>
         <v>2.6870231758453751</v>
       </c>
       <c r="V15" s="1">
-        <f>SUM(V2:V14)</f>
+        <f t="shared" si="0"/>
         <v>2.7504161816247565</v>
       </c>
       <c r="W15" s="1">
-        <f>SUM(W2:W14)</f>
+        <f t="shared" si="0"/>
         <v>2.7669346857220454</v>
       </c>
       <c r="X15" s="1">
-        <f>SUM(X2:X14)</f>
+        <f t="shared" si="0"/>
         <v>2.7517506159754279</v>
       </c>
       <c r="Y15" s="1">
-        <f>SUM(Y2:Y14)</f>
+        <f t="shared" si="0"/>
         <v>2.7588975372138957</v>
       </c>
       <c r="Z15" s="1">
-        <f>SUM(Z2:Z14)</f>
+        <f t="shared" si="0"/>
         <v>2.8000008004914734</v>
       </c>
       <c r="AA15" s="1">
-        <f>SUM(AA2:AA14)</f>
+        <f t="shared" si="0"/>
         <v>2.7897354851259424</v>
       </c>
       <c r="AB15" s="1">
-        <f>SUM(AB2:AB14)</f>
+        <f t="shared" si="0"/>
         <v>2.7276194096066746</v>
       </c>
       <c r="AC15" s="1">
-        <f>SUM(AC2:AC14)</f>
+        <f t="shared" si="0"/>
         <v>2.6872755890998681</v>
       </c>
       <c r="AD15" s="1">
-        <f>SUM(AD2:AD14)</f>
+        <f t="shared" si="0"/>
         <v>2.6594118253321049</v>
       </c>
       <c r="AE15" s="1">
-        <f>SUM(AE2:AE14)</f>
+        <f t="shared" si="0"/>
         <v>2.6709004618721846</v>
       </c>
       <c r="AF15" s="1">
-        <f>SUM(AF2:AF14)</f>
+        <f t="shared" si="0"/>
         <v>2.6539619689429865</v>
       </c>
     </row>
@@ -3340,7 +3367,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:AJ14"/>
+  <dimension ref="A1:AJ16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.5546875" customWidth="1"/>
@@ -3463,7 +3490,7 @@
         <v>36</v>
       </c>
       <c r="B2" s="21">
-        <f>_xlfn.MODE.SNGL(F2:AJ2)</f>
+        <f t="shared" ref="B2:B14" si="0">_xlfn.MODE.SNGL(F2:AJ2)</f>
         <v>1</v>
       </c>
       <c r="C2" s="22">
@@ -3577,19 +3604,19 @@
         <v>38</v>
       </c>
       <c r="B3" s="21">
-        <f>_xlfn.MODE.SNGL(F3:AJ3)</f>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="C3" s="22">
-        <f t="shared" ref="C3:C14" si="0">_xlfn.MODE.SNGL(F3:I3)</f>
+        <f t="shared" ref="C3:C14" si="1">_xlfn.MODE.SNGL(F3:I3)</f>
         <v>2</v>
       </c>
       <c r="D3" s="22">
-        <f t="shared" ref="D3:D14" si="1">_xlfn.MODE.SNGL(J3:U3)</f>
+        <f t="shared" ref="D3:D14" si="2">_xlfn.MODE.SNGL(J3:U3)</f>
         <v>2</v>
       </c>
       <c r="E3" s="23">
-        <f t="shared" ref="E3:E14" si="2">_xlfn.MODE.SNGL(V3:AJ3)</f>
+        <f t="shared" ref="E3:E14" si="3">_xlfn.MODE.SNGL(V3:AJ3)</f>
         <v>2</v>
       </c>
       <c r="F3" s="6">
@@ -3691,19 +3718,19 @@
         <v>35</v>
       </c>
       <c r="B4" s="21">
-        <f>_xlfn.MODE.SNGL(F4:AJ4)</f>
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="C4" s="24">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>6</v>
       </c>
       <c r="D4" s="24">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>5</v>
       </c>
       <c r="E4" s="23">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>3</v>
       </c>
       <c r="F4" s="6">
@@ -3805,19 +3832,19 @@
         <v>43</v>
       </c>
       <c r="B5" s="21">
-        <f>_xlfn.MODE.SNGL(F5:AJ5)</f>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="C5" s="24">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>9</v>
       </c>
       <c r="D5" s="22">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>4</v>
       </c>
       <c r="E5" s="23">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>4</v>
       </c>
       <c r="F5" s="6">
@@ -3919,19 +3946,19 @@
         <v>37</v>
       </c>
       <c r="B6" s="21">
-        <f>_xlfn.MODE.SNGL(F6:AJ6)</f>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="C6" s="24">
-        <f t="shared" si="0"/>
-        <v>3</v>
-      </c>
-      <c r="D6" s="24">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
+      <c r="D6" s="24">
+        <f t="shared" si="2"/>
+        <v>3</v>
+      </c>
       <c r="E6" s="23">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>5</v>
       </c>
       <c r="F6" s="6">
@@ -4033,15 +4060,15 @@
         <v>40</v>
       </c>
       <c r="B7" s="21">
-        <f>_xlfn.MODE.SNGL(F7:AJ7)</f>
+        <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="C7" s="24">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
       <c r="D7" s="22">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>6</v>
       </c>
       <c r="E7" s="23">
@@ -4147,19 +4174,19 @@
         <v>39</v>
       </c>
       <c r="B8" s="21">
-        <f>_xlfn.MODE.SNGL(F8:AJ8)</f>
-        <v>7</v>
-      </c>
-      <c r="C8" s="22">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="D8" s="22">
+      <c r="C8" s="22">
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
+      <c r="D8" s="22">
+        <f t="shared" si="2"/>
+        <v>7</v>
+      </c>
       <c r="E8" s="25">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>10</v>
       </c>
       <c r="F8" s="6">
@@ -4261,19 +4288,19 @@
         <v>32</v>
       </c>
       <c r="B9" s="21">
-        <f>_xlfn.MODE.SNGL(F9:AJ9)</f>
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="C9" s="24">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>11</v>
       </c>
       <c r="D9" s="24">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>10</v>
       </c>
       <c r="E9" s="23">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>8</v>
       </c>
       <c r="F9" s="6">
@@ -4375,19 +4402,19 @@
         <v>41</v>
       </c>
       <c r="B10" s="21">
-        <f>_xlfn.MODE.SNGL(F10:AJ10)</f>
-        <v>9</v>
-      </c>
-      <c r="C10" s="22">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="D10" s="22">
+      <c r="C10" s="22">
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
+      <c r="D10" s="22">
+        <f t="shared" si="2"/>
+        <v>9</v>
+      </c>
       <c r="E10" s="23">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>9</v>
       </c>
       <c r="F10" s="6">
@@ -4489,19 +4516,19 @@
         <v>33</v>
       </c>
       <c r="B11" s="21">
-        <f>_xlfn.MODE.SNGL(F11:AJ11)</f>
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="C11" s="24">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="D11" s="22">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>10</v>
       </c>
       <c r="E11" s="26">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>11</v>
       </c>
       <c r="F11" s="6">
@@ -4603,19 +4630,19 @@
         <v>44</v>
       </c>
       <c r="B12" s="21">
-        <f>_xlfn.MODE.SNGL(F12:AJ12)</f>
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
       <c r="C12" s="27">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>10</v>
       </c>
       <c r="D12" s="22">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>11</v>
       </c>
       <c r="E12" s="25">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>7</v>
       </c>
       <c r="F12" s="6">
@@ -4717,19 +4744,19 @@
         <v>42</v>
       </c>
       <c r="B13" s="21">
-        <f>_xlfn.MODE.SNGL(F13:AJ13)</f>
-        <v>12</v>
-      </c>
-      <c r="C13" s="22">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="D13" s="22">
+      <c r="C13" s="22">
         <f t="shared" si="1"/>
         <v>12</v>
       </c>
+      <c r="D13" s="22">
+        <f t="shared" si="2"/>
+        <v>12</v>
+      </c>
       <c r="E13" s="23">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>12</v>
       </c>
       <c r="F13" s="6">
@@ -4831,21 +4858,21 @@
         <v>34</v>
       </c>
       <c r="B14" s="28">
-        <f>_xlfn.MODE.SNGL(F14:AJ14)</f>
-        <v>13</v>
-      </c>
-      <c r="C14" s="29">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="D14" s="29">
+      <c r="C14" s="29">
         <f t="shared" si="1"/>
         <v>13</v>
       </c>
-      <c r="E14" s="30">
+      <c r="D14" s="29">
         <f t="shared" si="2"/>
         <v>13</v>
       </c>
+      <c r="E14" s="30">
+        <f t="shared" si="3"/>
+        <v>13</v>
+      </c>
       <c r="F14" s="9">
         <v>10</v>
       </c>
@@ -4938,6 +4965,101 @@
       </c>
       <c r="AJ14" s="11">
         <v>13</v>
+      </c>
+    </row>
+    <row r="16" spans="1:36" x14ac:dyDescent="0.3">
+      <c r="F16" s="32">
+        <v>1</v>
+      </c>
+      <c r="G16" s="32">
+        <v>2</v>
+      </c>
+      <c r="H16" s="32">
+        <v>3</v>
+      </c>
+      <c r="I16" s="32">
+        <v>4</v>
+      </c>
+      <c r="J16" s="31">
+        <v>1</v>
+      </c>
+      <c r="K16" s="31">
+        <v>2</v>
+      </c>
+      <c r="L16" s="31">
+        <v>3</v>
+      </c>
+      <c r="M16" s="31">
+        <v>4</v>
+      </c>
+      <c r="N16" s="31">
+        <v>5</v>
+      </c>
+      <c r="O16" s="31">
+        <v>6</v>
+      </c>
+      <c r="P16" s="31">
+        <v>7</v>
+      </c>
+      <c r="Q16" s="31">
+        <v>8</v>
+      </c>
+      <c r="R16" s="31">
+        <v>9</v>
+      </c>
+      <c r="S16" s="31">
+        <v>10</v>
+      </c>
+      <c r="T16" s="31">
+        <v>11</v>
+      </c>
+      <c r="U16" s="31">
+        <v>12</v>
+      </c>
+      <c r="V16" s="33">
+        <v>1</v>
+      </c>
+      <c r="W16" s="33">
+        <v>2</v>
+      </c>
+      <c r="X16" s="33">
+        <v>3</v>
+      </c>
+      <c r="Y16" s="33">
+        <v>4</v>
+      </c>
+      <c r="Z16" s="33">
+        <v>5</v>
+      </c>
+      <c r="AA16" s="33">
+        <v>6</v>
+      </c>
+      <c r="AB16" s="33">
+        <v>7</v>
+      </c>
+      <c r="AC16" s="33">
+        <v>8</v>
+      </c>
+      <c r="AD16" s="33">
+        <v>9</v>
+      </c>
+      <c r="AE16" s="33">
+        <v>10</v>
+      </c>
+      <c r="AF16" s="33">
+        <v>11</v>
+      </c>
+      <c r="AG16" s="33">
+        <v>12</v>
+      </c>
+      <c r="AH16" s="33">
+        <v>13</v>
+      </c>
+      <c r="AI16" s="33">
+        <v>14</v>
+      </c>
+      <c r="AJ16" s="33">
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>